<commit_message>
Version 1.6.0: Umrichter SINAMICS G120, Vor-Ort-Steuerstelle -S50, Tiefenschatten
- Band 1, Band 2, Rollenkurve und Pruefband wahlweise an Frequenzumrichtern -TA2...-TA5
  (Standardtelegramm 1, %QW/%IW256...270) statt an Schuetzen, fuer TO_SpeedAxis wie an echten G120
- PROFIdrive-Zustandsmaschine mit AUS1/AUS2/AUS3, Hochlaufgeber, STO ueber Not-Halt,
  Stoerungen F30005/F07011, HAND-Betrieb ueber das Bedienpanel IOP-2
- Vier G120 im Schaltschrank mit Live-Display und LEDs; Fenster "Umrichter" mit bedienbarem
  Panel, Telegramm Bit fuer Bit und Rampen live
- Vor-Ort-Steuerstelle -S50 am Pruefband mit Drehzahlpotentiometer (%IW70)
- Zuschaltbare Tiefenschatten (GTAO aus three.js r170)
- Rohre, Schlaeuche und Kabel mit richtigem Umlaufsinn
- Signalliste, TIA-Variablentabellen, Doku und alle Doku-Bilder aktualisiert,
  neues Werkzeug tools/doku-bilder.mjs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TIA/PLC_Tags_Tinning_EN.xlsx
+++ b/TIA/PLC_Tags_Tinning_EN.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J135"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6096,6 +6096,888 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>TA2_STW1</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>%QW256</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>-TA2 conveyor motor drive: control word 1 STW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>TA2_NSOLL_A</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>%QW258</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>-TA2 conveyor motor drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 100 mm/s)</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>TA2_ZSW1</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>%IW256</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>-TA2 conveyor motor drive: status word 1 ZSW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>TA2_NIST_A</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>%IW258</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>-TA2 conveyor motor drive: actual speed NIST_A (16#4000 = 1500 rpm = 100 mm/s)</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>TA3_STW1</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>%QW260</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>-TA3 conveyor 2 drive: control word 1 STW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>TA3_NSOLL_A</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>%QW262</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>-TA3 conveyor 2 drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 120 mm/s)</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>TA3_ZSW1</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>%IW260</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>-TA3 conveyor 2 drive: status word 1 ZSW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>TA3_NIST_A</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>%IW262</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>-TA3 conveyor 2 drive: actual speed NIST_A (16#4000 = 1500 rpm = 120 mm/s)</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>TA4_STW1</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>%QW264</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>-TA4 roller curve drive: control word 1 STW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>TA4_NSOLL_A</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>%QW266</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>-TA4 roller curve drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 110 mm/s)</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>TA4_ZSW1</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>%IW264</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>-TA4 roller curve drive: status word 1 ZSW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>TA4_NIST_A</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>%IW266</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>-TA4 roller curve drive: actual speed NIST_A (16#4000 = 1500 rpm = 110 mm/s)</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>TA5_STW1</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>%QW268</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>-TA5 inspection conveyor drive: control word 1 STW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>TA5_NSOLL_A</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>%QW270</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>-TA5 inspection conveyor drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 150 mm/s)</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>TA5_ZSW1</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>%IW268</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>-TA5 inspection conveyor drive: status word 1 ZSW1 (standard telegram 1)</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>TA5_NIST_A</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>%IW270</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>-TA5 inspection conveyor drive: actual speed NIST_A (16#4000 = 1500 rpm = 150 mm/s)</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>SA7_Local5</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>%I11.2</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Key switch local control station inspection conveyor -S50 (1 = local)</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>SF45_InspConv_On</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>%I11.3</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Local -S50 inspection conveyor ON (NO contact)</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>SF46_InspConv_Off</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>%I11.4</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Local -S50 inspection conveyor OFF (NC contact: 1 = not pressed)</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>SF47_InspConv_Speed</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>%IW70</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Local -S50 speed potentiometer inspection conveyor 0...27648 = 0...100 %</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>PF16_Local5</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>%Q5.3</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Lamp local control station inspection conveyor -S50 active</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Version 1.7.0: Füllstandsmessung und Nachspeisung des Kühlwassertanks
- Micropilot FMR20B -BL2 (Radar, stetig), Liquiphant FTL31 -BG38 MIN und -BG39 MAX (Ruhestrom)
- Nachspeisung über Magnetventil -MB17 und Regelventil -MB18 mit Stellungsrückmeldung
- Übungsumfang Kühlwassertank: Niveauregler automatisch oder SPS regelt (Demo-SPS mit PI-Regler)
- Ablasshahn als Störgröße, Trockenlauf der Pumpe -MA3, AQ-4-Baugruppe im Schaltschrank
- 6 neue Signale (161), TIA-Tabellen, Doku mit Übungen 21-24, Bild 14-kuehlwassertank

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TIA/PLC_Tags_Tinning_EN.xlsx
+++ b/TIA/PLC_Tags_Tinning_EN.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6978,6 +6978,258 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>MB17_WaterRefill</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>%Q5.4</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>-MB17 fresh water solenoid valve cooling water tank: refill (2/2 NC, in series with control valve -MB18)</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>MB18_ControlValve</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>%QW80</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>-MB18 fresh water control valve: setpoint 0...27648 = 0...100 % (AQ 4 channel 0, stroke time 8 s)</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>MB18_ValvePosition</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>%IW74</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>-MB18 control valve: position feedback 0...27648 = 0...100 %</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>BL2_WaterLevel</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Int</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>%IW72</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>-BL2 cooling water tank level, radar Micropilot FMR20B: 0...27648 = 0...100 %</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>BG38_Water_Min</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>%I11.5</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>-BG38 point level switch Liquiphant FTL31 cooling water tank MIN (1 = fork covered, above 25 %, dry-run protection -MA3)</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>BG39_Water_Max_free</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>%I11.6</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>-BG39 point level switch Liquiphant FTL31 cooling water tank MAX (1 = fork free, below 90 %; 0 = full or wire break)</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Version 1.8.0: Abfrage "Korb liegt am Anschlag" -BG40
- -BG11 meldet den Korb schon 55 mm vor dem Anschlag -MM5, die Zeit bis zum
  Anliegen haengt von der Bandgeschwindigkeit ab
- Gefederte Anschlagleiste an -MM5/-MM6 (Resthub 3 mm gegen den Daempfer),
  Schaltfahne und induktiver Sensor M8 -BG40 auf dem Hebel von -MM5
- BG40_Korb_am_Anschlag %I8.0, Leitung ueber die Drehachse zu -XD3 X4
- Demo-SPS startet mit -BG40 statt 1,5 s nach -BG11, PF4 und HMI zeigen -BG40
- 162 Signale, TIA-Tabellen, Doku, Uebung 7 mit Einlaufueberwachung

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TIA/PLC_Tags_Tinning_EN.xlsx
+++ b/TIA/PLC_Tags_Tinning_EN.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Light barrier material basket at transfer position</t>
+          <t>Light barrier transfer point inlet (basket arriving, not yet resting against the stop)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4923,7 +4923,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SF28_MM8_Tip</t>
+          <t>BG40_Basket_at_Stop</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -4938,12 +4938,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>%I8.2</t>
+          <t>%I8.0</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Manual button -MM8 tip tipper</t>
+          <t>Basket resting against stop -MM5 (inductive M8 sensor on the spring-loaded stop bar)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -4965,7 +4965,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SF29_MM8_Return</t>
+          <t>SF28_MM8_Tip</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -4980,12 +4980,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>%I8.3</t>
+          <t>%I8.2</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Manual button -MM8 tipper back</t>
+          <t>Manual button -MM8 tip tipper</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5007,7 +5007,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SA5_Local3</t>
+          <t>SF29_MM8_Return</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5022,12 +5022,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>%I8.4</t>
+          <t>%I8.3</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Key switch local control station -S30 (1 = active)</t>
+          <t>Manual button -MM8 tipper back</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5049,7 +5049,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SF30_Curve_Fwd</t>
+          <t>SA5_Local3</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5064,12 +5064,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>%I8.5</t>
+          <t>%I8.4</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Local roller curve forward (NO contact)</t>
+          <t>Key switch local control station -S30 (1 = active)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5091,7 +5091,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SF31_Curve_Rev</t>
+          <t>SF30_Curve_Fwd</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5106,12 +5106,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>%I8.6</t>
+          <t>%I8.5</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Local roller curve reverse (NO contact)</t>
+          <t>Local roller curve forward (NO contact)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5133,7 +5133,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SF32_Curve_Halt</t>
+          <t>SF31_Curve_Rev</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5148,12 +5148,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>%I8.7</t>
+          <t>%I8.6</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Local roller curve stop (NC contact: 1 = not pressed)</t>
+          <t>Local roller curve reverse (NO contact)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5175,7 +5175,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FA7_MotorProtection3</t>
+          <t>SF32_Curve_Halt</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5190,12 +5190,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>%I9.0</t>
+          <t>%I8.7</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Motor protection switch roller curve -FA7, auxiliary contact (1 = OK)</t>
+          <t>Local roller curve stop (NC contact: 1 = not pressed)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -5217,7 +5217,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SF0_EStop_Released</t>
+          <t>FA7_MotorProtection3</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5232,12 +5232,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>%I9.1</t>
+          <t>%I9.0</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>E-stop -SF0 operator panel, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
+          <t>Motor protection switch roller curve -FA7, auxiliary contact (1 = OK)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5259,7 +5259,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SF8_EStop_Released</t>
+          <t>SF0_EStop_Released</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5274,12 +5274,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>%I9.2</t>
+          <t>%I9.1</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>E-stop -SF8 local -S10 conveyor 1, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
+          <t>E-stop -SF0 operator panel, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -5301,7 +5301,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SF9_EStop_Released</t>
+          <t>SF8_EStop_Released</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5316,12 +5316,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>%I9.3</t>
+          <t>%I9.2</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>E-stop -SF9 local -S20 conveyor 2, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
+          <t>E-stop -SF8 local -S10 conveyor 1, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -5343,7 +5343,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SF10_EStop_Released</t>
+          <t>SF9_EStop_Released</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5358,12 +5358,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>%I9.4</t>
+          <t>%I9.3</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>E-stop -SF10 local -S30 roller curve, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
+          <t>E-stop -SF9 local -S20 conveyor 2, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5385,7 +5385,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SF33_EStop_Released</t>
+          <t>SF10_EStop_Released</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5400,12 +5400,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>%I9.5</t>
+          <t>%I9.4</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>E-stop -SF33 local -S40 inspection station, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
+          <t>E-stop -SF10 local -S30 roller curve, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5427,7 +5427,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SA6_Local4</t>
+          <t>SF33_EStop_Released</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -5442,12 +5442,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>%I9.6</t>
+          <t>%I9.5</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Key switch local control station -S40 (1 = active, station automatic paused)</t>
+          <t>E-stop -SF33 local -S40 inspection station, signaling contact (NC contact: 1 = released, 0 = pressed)</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5469,7 +5469,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SF34_Insp_On</t>
+          <t>SA6_Local4</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -5484,12 +5484,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>%I9.7</t>
+          <t>%I9.6</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Local -S40 vibratory chute + inspection conveyor ON (NO contact, latching in the PLC)</t>
+          <t>Key switch local control station -S40 (1 = active, station automatic paused)</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5511,7 +5511,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SF35_Insp_Off</t>
+          <t>SF34_Insp_On</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -5526,12 +5526,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>%I10.0</t>
+          <t>%I9.7</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Local -S40 vibratory chute + inspection conveyor OFF (NC contact: 1 = not pressed)</t>
+          <t>Local -S40 vibratory chute + inspection conveyor ON (NO contact, latching in the PLC)</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5553,7 +5553,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SF36_Trough_Fwd</t>
+          <t>SF35_Insp_Off</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -5568,12 +5568,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>%I10.1</t>
+          <t>%I10.0</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Local -S40 jog trough rollers forward (NO contact)</t>
+          <t>Local -S40 vibratory chute + inspection conveyor OFF (NC contact: 1 = not pressed)</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -5595,7 +5595,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SF37_Trough_Rev</t>
+          <t>SF36_Trough_Fwd</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -5610,12 +5610,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>%I10.2</t>
+          <t>%I10.1</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Local -S40 jog trough rollers backward (NO contact)</t>
+          <t>Local -S40 jog trough rollers forward (NO contact)</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -5637,7 +5637,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SF38_Tipper_Tip</t>
+          <t>SF37_Trough_Rev</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5652,12 +5652,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>%I10.3</t>
+          <t>%I10.2</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Local -S40 tip tipper (NO contact, only with basket at -BG33 or empty trough)</t>
+          <t>Local -S40 jog trough rollers backward (NO contact)</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -5679,7 +5679,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SF39_Tipper_Return</t>
+          <t>SF38_Tipper_Tip</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -5694,12 +5694,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>%I10.4</t>
+          <t>%I10.3</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Local -S40 tipper back (NO contact)</t>
+          <t>Local -S40 tip tipper (NO contact, only with basket at -BG33 or empty trough)</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -5721,7 +5721,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>FA8_MotorProtection4</t>
+          <t>SF39_Tipper_Return</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5736,12 +5736,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>%I10.5</t>
+          <t>%I10.4</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Motor protection switch trough drive -MA7 -FA8, auxiliary contact (1 = OK)</t>
+          <t>Local -S40 tipper back (NO contact)</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -5763,7 +5763,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SF41_Ack_S10</t>
+          <t>FA8_MotorProtection4</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -5778,12 +5778,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>%I10.6</t>
+          <t>%I10.5</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Acknowledge button local -S10 conveyor 1 (NO contact, parallel to -SF4 on -KF2)</t>
+          <t>Motor protection switch trough drive -MA7 -FA8, auxiliary contact (1 = OK)</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -5805,7 +5805,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SF42_Ack_S20</t>
+          <t>SF41_Ack_S10</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5820,12 +5820,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>%I10.7</t>
+          <t>%I10.6</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Acknowledge button local -S20 conveyor 2 (NO contact, parallel to -SF4 on -KF2)</t>
+          <t>Acknowledge button local -S10 conveyor 1 (NO contact, parallel to -SF4 on -KF2)</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -5847,7 +5847,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SF43_Ack_S30</t>
+          <t>SF42_Ack_S20</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -5862,12 +5862,12 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>%I11.0</t>
+          <t>%I10.7</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Acknowledge button local -S30 roller curve (NO contact, parallel to -SF4 on -KF2)</t>
+          <t>Acknowledge button local -S20 conveyor 2 (NO contact, parallel to -SF4 on -KF2)</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -5889,7 +5889,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SF44_Ack_S40</t>
+          <t>SF43_Ack_S30</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -5904,12 +5904,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>%I11.1</t>
+          <t>%I11.0</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Acknowledge button local -S40 inspection station (NO contact, parallel to -SF4 on -KF2)</t>
+          <t>Acknowledge button local -S30 roller curve (NO contact, parallel to -SF4 on -KF2)</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -5931,7 +5931,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>BT1_TinTemperature</t>
+          <t>SF44_Ack_S40</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -5941,17 +5941,17 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Bool</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>%IW64</t>
+          <t>%I11.1</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Tin temperature analog 0...27648 = 0...400 deg C</t>
+          <t>Acknowledge button local -S40 inspection station (NO contact, parallel to -SF4 on -KF2)</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -5973,7 +5973,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>BL1_FillLevel</t>
+          <t>BT1_TinTemperature</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -5988,12 +5988,12 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>%IW66</t>
+          <t>%IW64</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Fill level analog 0...27648 = 0...100 %</t>
+          <t>Tin temperature analog 0...27648 = 0...400 deg C</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -6015,7 +6015,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>BT2_BasketTemperature</t>
+          <t>BL1_FillLevel</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -6030,12 +6030,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>%IW68</t>
+          <t>%IW66</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Pyrometer cooling station: basket temperature 0...27648 = 0...400 deg C</t>
+          <t>Fill level analog 0...27648 = 0...100 %</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -6057,7 +6057,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>BG37_Tipper_Inlet</t>
+          <t>BT2_BasketTemperature</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6067,17 +6067,17 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Bool</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>%I11.7</t>
+          <t>%IW68</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Light barrier tipping trough inlet (basket in trough, swivels with it)</t>
+          <t>Pyrometer cooling station: basket temperature 0...27648 = 0...400 deg C</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -6099,7 +6099,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>TA2_STW1</t>
+          <t>BG37_Tipper_Inlet</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -6109,17 +6109,17 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Bool</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>%QW256</t>
+          <t>%I11.7</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>-TA2 conveyor motor drive: control word 1 STW1 (standard telegram 1)</t>
+          <t>Light barrier tipping trough inlet (basket in trough, swivels with it)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -6141,7 +6141,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>TA2_NSOLL_A</t>
+          <t>TA2_STW1</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6151,17 +6151,17 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>%QW258</t>
+          <t>%QW256</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>-TA2 conveyor motor drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 100 mm/s)</t>
+          <t>-TA2 conveyor motor drive: control word 1 STW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -6183,7 +6183,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>TA2_ZSW1</t>
+          <t>TA2_NSOLL_A</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -6193,17 +6193,17 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>%IW256</t>
+          <t>%QW258</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>-TA2 conveyor motor drive: status word 1 ZSW1 (standard telegram 1)</t>
+          <t>-TA2 conveyor motor drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 100 mm/s)</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -6225,7 +6225,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>TA2_NIST_A</t>
+          <t>TA2_ZSW1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6235,17 +6235,17 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>%IW258</t>
+          <t>%IW256</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>-TA2 conveyor motor drive: actual speed NIST_A (16#4000 = 1500 rpm = 100 mm/s)</t>
+          <t>-TA2 conveyor motor drive: status word 1 ZSW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6267,7 +6267,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>TA3_STW1</t>
+          <t>TA2_NIST_A</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -6277,17 +6277,17 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>%QW260</t>
+          <t>%IW258</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>-TA3 conveyor 2 drive: control word 1 STW1 (standard telegram 1)</t>
+          <t>-TA2 conveyor motor drive: actual speed NIST_A (16#4000 = 1500 rpm = 100 mm/s)</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -6309,7 +6309,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>TA3_NSOLL_A</t>
+          <t>TA3_STW1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6319,17 +6319,17 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>%QW262</t>
+          <t>%QW260</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>-TA3 conveyor 2 drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 120 mm/s)</t>
+          <t>-TA3 conveyor 2 drive: control word 1 STW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -6351,7 +6351,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>TA3_ZSW1</t>
+          <t>TA3_NSOLL_A</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -6361,17 +6361,17 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>%IW260</t>
+          <t>%QW262</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>-TA3 conveyor 2 drive: status word 1 ZSW1 (standard telegram 1)</t>
+          <t>-TA3 conveyor 2 drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 120 mm/s)</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -6393,7 +6393,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>TA3_NIST_A</t>
+          <t>TA3_ZSW1</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -6403,17 +6403,17 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>%IW262</t>
+          <t>%IW260</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>-TA3 conveyor 2 drive: actual speed NIST_A (16#4000 = 1500 rpm = 120 mm/s)</t>
+          <t>-TA3 conveyor 2 drive: status word 1 ZSW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -6435,7 +6435,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>TA4_STW1</t>
+          <t>TA3_NIST_A</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -6445,17 +6445,17 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>%QW264</t>
+          <t>%IW262</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>-TA4 roller curve drive: control word 1 STW1 (standard telegram 1)</t>
+          <t>-TA3 conveyor 2 drive: actual speed NIST_A (16#4000 = 1500 rpm = 120 mm/s)</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -6477,7 +6477,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>TA4_NSOLL_A</t>
+          <t>TA4_STW1</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -6487,17 +6487,17 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>%QW266</t>
+          <t>%QW264</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>-TA4 roller curve drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 110 mm/s)</t>
+          <t>-TA4 roller curve drive: control word 1 STW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -6519,7 +6519,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>TA4_ZSW1</t>
+          <t>TA4_NSOLL_A</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -6529,17 +6529,17 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>%IW264</t>
+          <t>%QW266</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>-TA4 roller curve drive: status word 1 ZSW1 (standard telegram 1)</t>
+          <t>-TA4 roller curve drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 110 mm/s)</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -6561,7 +6561,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>TA4_NIST_A</t>
+          <t>TA4_ZSW1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -6571,17 +6571,17 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>%IW266</t>
+          <t>%IW264</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>-TA4 roller curve drive: actual speed NIST_A (16#4000 = 1500 rpm = 110 mm/s)</t>
+          <t>-TA4 roller curve drive: status word 1 ZSW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -6603,7 +6603,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>TA5_STW1</t>
+          <t>TA4_NIST_A</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -6613,17 +6613,17 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>%QW268</t>
+          <t>%IW266</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>-TA5 inspection conveyor drive: control word 1 STW1 (standard telegram 1)</t>
+          <t>-TA4 roller curve drive: actual speed NIST_A (16#4000 = 1500 rpm = 110 mm/s)</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -6645,7 +6645,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>TA5_NSOLL_A</t>
+          <t>TA5_STW1</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6655,17 +6655,17 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>%QW270</t>
+          <t>%QW268</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>-TA5 inspection conveyor drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 150 mm/s)</t>
+          <t>-TA5 inspection conveyor drive: control word 1 STW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -6687,7 +6687,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>TA5_ZSW1</t>
+          <t>TA5_NSOLL_A</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -6697,17 +6697,17 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Word</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>%IW268</t>
+          <t>%QW270</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>-TA5 inspection conveyor drive: status word 1 ZSW1 (standard telegram 1)</t>
+          <t>-TA5 inspection conveyor drive: speed setpoint NSOLL_A (16#4000 = 1500 rpm = 150 mm/s)</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6729,7 +6729,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>TA5_NIST_A</t>
+          <t>TA5_ZSW1</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -6739,17 +6739,17 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Word</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>%IW270</t>
+          <t>%IW268</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>-TA5 inspection conveyor drive: actual speed NIST_A (16#4000 = 1500 rpm = 150 mm/s)</t>
+          <t>-TA5 inspection conveyor drive: status word 1 ZSW1 (standard telegram 1)</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -6771,7 +6771,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SA7_Local5</t>
+          <t>TA5_NIST_A</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -6781,17 +6781,17 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Bool</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>%I11.2</t>
+          <t>%IW270</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Key switch local control station inspection conveyor -S50 (1 = local)</t>
+          <t>-TA5 inspection conveyor drive: actual speed NIST_A (16#4000 = 1500 rpm = 150 mm/s)</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -6813,7 +6813,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SF45_InspConv_On</t>
+          <t>SA7_Local5</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -6828,12 +6828,12 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>%I11.3</t>
+          <t>%I11.2</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Local -S50 inspection conveyor ON (NO contact)</t>
+          <t>Key switch local control station inspection conveyor -S50 (1 = local)</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -6855,7 +6855,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SF46_InspConv_Off</t>
+          <t>SF45_InspConv_On</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -6870,12 +6870,12 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>%I11.4</t>
+          <t>%I11.3</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Local -S50 inspection conveyor OFF (NC contact: 1 = not pressed)</t>
+          <t>Local -S50 inspection conveyor ON (NO contact)</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -6897,7 +6897,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>SF47_InspConv_Speed</t>
+          <t>SF46_InspConv_Off</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -6907,17 +6907,17 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Bool</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>%IW70</t>
+          <t>%I11.4</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Local -S50 speed potentiometer inspection conveyor 0...27648 = 0...100 %</t>
+          <t>Local -S50 inspection conveyor OFF (NC contact: 1 = not pressed)</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -6939,7 +6939,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PF16_Local5</t>
+          <t>SF47_InspConv_Speed</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -6949,17 +6949,17 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Bool</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>%Q5.3</t>
+          <t>%IW70</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Lamp local control station inspection conveyor -S50 active</t>
+          <t>Local -S50 speed potentiometer inspection conveyor 0...27648 = 0...100 %</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6981,7 +6981,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>MB17_WaterRefill</t>
+          <t>PF16_Local5</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>%Q5.4</t>
+          <t>%Q5.3</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>-MB17 fresh water solenoid valve cooling water tank: refill (2/2 NC, in series with control valve -MB18)</t>
+          <t>Lamp local control station inspection conveyor -S50 active</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -7023,7 +7023,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MB18_ControlValve</t>
+          <t>MB17_WaterRefill</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -7033,17 +7033,17 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>Bool</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>%QW80</t>
+          <t>%Q5.4</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>-MB18 fresh water control valve: setpoint 0...27648 = 0...100 % (AQ 4 channel 0, stroke time 8 s)</t>
+          <t>-MB17 fresh water solenoid valve cooling water tank: refill (2/2 NC, in series with control valve -MB18)</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -7065,7 +7065,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MB18_ValvePosition</t>
+          <t>MB18_ControlValve</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -7080,12 +7080,12 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>%IW74</t>
+          <t>%QW80</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>-MB18 control valve: position feedback 0...27648 = 0...100 %</t>
+          <t>-MB18 fresh water control valve: setpoint 0...27648 = 0...100 % (AQ 4 channel 0, stroke time 8 s)</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -7107,7 +7107,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>BL2_WaterLevel</t>
+          <t>MB18_ValvePosition</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -7122,12 +7122,12 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>%IW72</t>
+          <t>%IW74</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>-BL2 cooling water tank level, radar Micropilot FMR20B: 0...27648 = 0...100 %</t>
+          <t>-MB18 control valve: position feedback 0...27648 = 0...100 %</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -7149,7 +7149,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>BG38_Water_Min</t>
+          <t>BL2_WaterLevel</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -7159,17 +7159,17 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Bool</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>%I11.5</t>
+          <t>%IW72</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>-BG38 point level switch Liquiphant FTL31 cooling water tank MIN (1 = fork covered, above 25 %, dry-run protection -MA3)</t>
+          <t>-BL2 cooling water tank level, radar Micropilot FMR20B: 0...27648 = 0...100 %</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -7191,40 +7191,82 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
+          <t>BG38_Water_Min</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>%I11.5</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>-BG38 point level switch Liquiphant FTL31 cooling water tank MIN (1 = fork covered, above 25 %, dry-run protection -MA3)</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
           <t>BG39_Water_Max_free</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>Tinning</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Bool</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
         <is>
           <t>%I11.6</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr">
+      <c r="E163" t="inlineStr">
         <is>
           <t>-BG39 point level switch Liquiphant FTL31 cooling water tank MAX (1 = fork free, below 90 %; 0 = full or wire break)</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr">
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
         <is>
           <t>True</t>
         </is>

</xml_diff>

<commit_message>
Version 1.9.0: Schwenkantrieb 90° an -MM5/-MM6, feste Anschlagleiste mit -BG40 (M12), Kollision Korbpuffer/Anschlag
- Anschlag und Vereinzeler mit pneumatischem Schwenkantrieb 90°, Endlagen über Schaltnocke
- Feste Anschlagleiste, -BG40 induktiv M12 bündig in der Leiste
- Vereinzeler 10 mm weiter zurück (Puffer kommt beim Anheben vorbei)
- Ablauf: Band stoppen, Anschlag öffnen, einhängen und anheben
- Kollision sichtbar: Korb kippt am Hebel, Abriss ab 10°, schiefes Aufsetzen
- Signaltexte, TIA-Tabellen, Doku, Bild 10-drosselventile

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TIA/PLC_Tags_Tinning_EN.xlsx
+++ b/TIA/PLC_Tags_Tinning_EN.xlsx
@@ -3641,7 +3641,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>-MM5 stop open</t>
+          <t>Stop -MM5 open (90 deg, only then lift or lower the basket)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Basket resting against stop -MM5 (inductive M8 sensor on the spring-loaded stop bar)</t>
+          <t>Basket resting against stop -MM5 (inductive M12 sensor flush in the stop bar)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">

</xml_diff>

<commit_message>
Version 1.14.0: Zwilling-Befunde aus dem Handbuch-Review, BCD-Geräte, Grafik
- Wiederanlaufsperre: automatische Bereiche nach Not-Halt erst mit START −SF1
- −KF2 gibt beim Loslassen des Quittiertasters frei (überwachter Start)
- Demo-SPS: Verriegelung −MM4 positiv, drahtbruchsicher
- Störgrößen Motorschutz −FA1/−FA5/−FA7/−FA8 und Drahtbruch an Analogwerten (7FFF)
- Signalmonitor: Dez/Hex/Bin, Byte-Zeilen
- G120: STW1.10 = 0 ignoriert Telegramm, F01910 mit AUS3, A07910 setzt ZSW1.7
- BCD-Anzeige −PG1 (%QW6) und Daumenradschalter −SF48 (%IW12), 4. DI-Baugruppe, 186 Signale
- Grafik: Hallenkulisse, HDR-Umgebung (CC0), Shader-Vorbereitung, weniger Dreiecke
- Handbuch, Schaltplan, Doku DE/EN und TIA-Variablentabellen nachgezogen

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TIA/PLC_Tags_Tinning_EN.xlsx
+++ b/TIA/PLC_Tags_Tinning_EN.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7272,6 +7272,1014 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_U1</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>%I13.0</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: units, weight 1 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_U2</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>%I13.1</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: units, weight 2 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_U4</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>%I13.2</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: units, weight 4 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_U8</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>%I13.3</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: units, weight 8 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_T1</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>%I13.4</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: tens, weight 1 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_T2</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>%I13.5</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: tens, weight 2 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_T4</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>%I13.6</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: tens, weight 4 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_T8</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>%I13.7</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: tens, weight 8 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_H1</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>%I12.0</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: hundreds, weight 1 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_H2</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>%I12.1</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: hundreds, weight 2 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_H4</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>%I12.2</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: hundreds, weight 4 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>SF48_DipTime_H8</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>%I12.3</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>-SF48 thumbwheel switch dip time: hundreds, weight 8 (as word %IW12 = BCD)</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>PG1_Display_U1</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>%Q7.0</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: units, weight 1 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>PG1_Display_U2</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>%Q7.1</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: units, weight 2 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>PG1_Display_U4</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>%Q7.2</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: units, weight 4 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>PG1_Display_U8</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>%Q7.3</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: units, weight 8 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>PG1_Display_T1</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>%Q7.4</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: tens, weight 1 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>PG1_Display_T2</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>%Q7.5</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: tens, weight 2 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>PG1_Display_T4</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>%Q7.6</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: tens, weight 4 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>PG1_Display_T8</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>%Q7.7</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: tens, weight 8 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>PG1_Display_H1</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>%Q6.0</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: hundreds, weight 1 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>PG1_Display_H2</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>%Q6.1</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: hundreds, weight 2 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>PG1_Display_H4</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>%Q6.2</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: hundreds, weight 4 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>PG1_Display_H8</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Tinning</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Bool</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>%Q6.3</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>-PG1 BCD display operator panel: hundreds, weight 8 (as word %QW6 = BCD)</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>